<commit_message>
update financial data files and fix their formats
</commit_message>
<xml_diff>
--- a/data/aura_motion_financial.xlsx
+++ b/data/aura_motion_financial.xlsx
@@ -2,23 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17640" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financial Model" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,74 +27,111 @@
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF1A237E"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color rgb="FF2D2D2D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF1A237E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <i val="1"/>
+      <color rgb="FF555555"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF1565C0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <i val="1"/>
+      <color rgb="FF888888"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF2D2D2D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <i val="1"/>
+      <color rgb="FF888888"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001A237E"/>
-      <sz val="11"/>
+      <color rgb="FF1A237E"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color theme="1"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="002D2D2D"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="001A237E"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FF2D2D2D"/>
       <sz val="12"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00555555"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="001565C0"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00888888"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="002D2D2D"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00888888"/>
-      <sz val="10"/>
+      <name val="Calibri"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="6">
@@ -107,26 +143,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001A237E"/>
+        <fgColor rgb="FF1A237E"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002D2D2D"/>
+        <fgColor rgb="FF2D2D2D"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF9C4"/>
+        <fgColor rgb="FFFFF9C4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8F5E9"/>
+        <fgColor rgb="FFE8F5E9"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -136,23 +172,68 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </left>
       <right style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </right>
       <top style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -166,45 +247,61 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -567,113 +664,180 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="90" customWidth="1" min="1" max="1"/>
+    <col width="21.42857142857143" customWidth="1" style="19" min="1" max="1"/>
+    <col width="107.1428571428571" customWidth="1" style="19" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
+    <row r="1" ht="40" customHeight="1" s="19">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">  Aura Motion 🎬 — Financial Model  |  Business Software Course · SRH Hochschule</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="22" customHeight="1" s="19">
+      <c r="A2" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  How to use this template</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="3" t="inlineStr"/>
-    </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="B2" s="22" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="22" t="n"/>
+      <c r="B3" s="22" t="n"/>
+    </row>
+    <row r="4" ht="18" customHeight="1" s="19">
+      <c r="A4" s="23" t="n"/>
+      <c r="B4" s="22" t="n"/>
+    </row>
+    <row r="5" ht="18" customHeight="1" s="19">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  🟦  BLUE cells</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>Pre-filled input values — these are given to you. Do not change them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1" s="19">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  🟨  YELLOW cells</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>Your task — write the correct Excel formula in each yellow cell. Each cell shows a hint describing what to calculate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1" s="19">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  🟩  GREEN cells</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="3" t="inlineStr"/>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>Auto-calculated results — formulas are already written. They update automatically once you fill in the yellow cells.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1" s="19">
+      <c r="A8" s="23" t="n"/>
+      <c r="B8" s="22" t="n"/>
+    </row>
+    <row r="9" ht="18" customHeight="1" s="19">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  Step 1</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>Open the 'Financial Model' tab (second sheet at the bottom of the screen).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="19">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  Step 2</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>Read row 3 — it explains the colour coding. Blue = given input, Yellow = write your formula, Green = auto-calculated result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1" s="19">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  Step 3</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
+        <is>
+          <t>Start with the REVENUE section (rows 5–9). Each yellow cell in column D shows a hint (e.g. '= Qty × Price'). Write the formula using the values in columns B and C on the same row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="19">
+      <c r="A12" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  Step 4</t>
         </is>
       </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="B12" s="24" t="inlineStr">
+        <is>
+          <t>Repeat for COST OF GOODS SOLD (rows 12–15) and FIXED COSTS (rows 22–26). The hints in each yellow cell tell you exactly what to calculate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="19">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  Step 5</t>
         </is>
       </c>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="3" t="inlineStr"/>
-    </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t>Check your results: does the Operating Profit look reasonable for this company? Compare it to the financial snapshot on your company portfolio page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="19">
+      <c r="A14" s="23" t="n"/>
+      <c r="B14" s="22" t="n"/>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="19">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  Tip</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="B15" s="24" t="inlineStr">
+        <is>
+          <t>A hint like '= Qty × Price' means: multiply the value in column B by column C on the same row. For row 5, that means typing =B5*C5 in cell D5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="19">
+      <c r="A16" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  Tip</t>
         </is>
       </c>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t>TOTAL rows (e.g. TOTAL REVENUE, TOTAL COGS) already have SUM formulas written in green — do not click into or overwrite them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1" s="19">
+      <c r="A17" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  Tip</t>
         </is>
       </c>
+      <c r="B17" s="24" t="inlineStr">
+        <is>
+          <t>If a hint says '= C × 12', the rate in column C is a monthly figure. Multiply by 12 to get the annual amount — e.g. =C22*12</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -685,488 +849,489 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E34"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" style="19" min="1" max="1"/>
+    <col width="18" customWidth="1" style="19" min="2" max="4"/>
+    <col width="8" customWidth="1" style="19" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="5" t="inlineStr">
+    <row r="1" ht="32" customHeight="1" s="19">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">  Aura Motion 🎬  |  Simplified P&amp;L Financial Model  |  FY 2025 (Projected)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="6" t="inlineStr">
+    <row r="2" ht="22" customHeight="1" s="19">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Line Item</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>Quantity / Driver</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>Unit Rate / Price</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>Amount (€)</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr"/>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="E2" s="5" t="n"/>
+    </row>
+    <row r="3" ht="18" customHeight="1" s="19">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">  🟦 Blue = given input  |  🟨 Yellow = write your formula here  |  🟩 Green = calculated result</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  1.  REVENUE</t>
         </is>
       </c>
+      <c r="B4" s="16" t="n"/>
+      <c r="C4" s="16" t="n"/>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="17" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">    Brand Animation projects  [Projects/year × Avg. Project Fee (€)]</t>
         </is>
       </c>
-      <c r="B5" s="10" t="n">
+      <c r="B5" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="C5" s="10" t="n">
+      <c r="C5" s="7" t="n">
         <v>4500</v>
       </c>
-      <c r="D5" s="11">
-        <f> Qty × Price</f>
+      <c r="D5" s="8">
+        <f>Qty * Price</f>
         <v/>
       </c>
-      <c r="E5" s="12" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">    Explainer Video projects  [Projects/year × Avg. Project Fee (€)]</t>
         </is>
       </c>
-      <c r="B6" s="10" t="n">
+      <c r="B6" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="C6" s="10" t="n">
+      <c r="C6" s="7" t="n">
         <v>3800</v>
       </c>
-      <c r="D6" s="11">
-        <f> Qty × Price</f>
+      <c r="D6" s="8">
+        <f>Qty * Price</f>
         <v/>
       </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">    Social Content retainers  [Retainer clients × Monthly Retainer (€)]</t>
         </is>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="C7" s="10" t="n">
+      <c r="C7" s="7" t="n">
         <v>1800</v>
       </c>
-      <c r="D7" s="11">
-        <f> Qty × Price</f>
+      <c r="D7" s="8">
+        <f>Qty * Price</f>
         <v/>
       </c>
-      <c r="E7" s="12" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">    Event Reels  [Projects/year × Avg. Project Fee (€)]</t>
         </is>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="7" t="n">
         <v>2200</v>
       </c>
-      <c r="D8" s="11">
-        <f> Qty × Price</f>
+      <c r="D8" s="8">
+        <f>Qty * Price</f>
         <v/>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">    TOTAL REVENUE</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr"/>
-      <c r="C9" s="14" t="inlineStr"/>
-      <c r="D9" s="11">
-        <f> SUM(D5:D8)</f>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="8">
+        <f>SUM(D5:D8)</f>
         <v/>
       </c>
-      <c r="E9" s="15" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="8" customHeight="1"/>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>€</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="8" customHeight="1" s="19"/>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  2.  COST OF GOODS SOLD  (Variable Costs)</t>
         </is>
       </c>
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="16" t="n"/>
+      <c r="D11" s="16" t="n"/>
+      <c r="E11" s="17" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">    Freelance animator cost per project</t>
         </is>
       </c>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>See projects above</t>
         </is>
       </c>
-      <c r="C12" s="10" t="n">
+      <c r="C12" s="7" t="n">
         <v>900</v>
       </c>
-      <c r="D12" s="11">
-        <f> Qty × Rate</f>
+      <c r="D12" s="8">
+        <f>Qty * Rate</f>
         <v/>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E12" s="9" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">    Stock footage &amp; assets per project</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>See projects above</t>
         </is>
       </c>
-      <c r="C13" s="10" t="n">
+      <c r="C13" s="7" t="n">
         <v>120</v>
       </c>
-      <c r="D13" s="11">
-        <f> Qty × Rate</f>
+      <c r="D13" s="8">
+        <f>Qty * Rate</f>
         <v/>
       </c>
-      <c r="E13" s="12" t="inlineStr">
+      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">    Software licenses (Adobe, DaVinci)</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>Annual cost ÷ 12</t>
         </is>
       </c>
-      <c r="C14" s="10" t="n">
+      <c r="C14" s="7" t="n">
         <v>210</v>
       </c>
-      <c r="D14" s="11">
-        <f> Rate × 12</f>
+      <c r="D14" s="8">
+        <f>Rate * 12</f>
         <v/>
       </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="E14" s="9" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">    TOTAL COGS</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr"/>
-      <c r="C15" s="14" t="inlineStr"/>
-      <c r="D15" s="11">
-        <f> SUM(D12:D14)</f>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="8">
+        <f>SUM(D12:D14)</f>
         <v/>
       </c>
-      <c r="E15" s="15" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="8" customHeight="1"/>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>€</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="8" customHeight="1" s="19"/>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  3.  GROSS PROFIT</t>
         </is>
       </c>
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="16" t="n"/>
+      <c r="D17" s="16" t="n"/>
+      <c r="E17" s="17" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">    Gross Profit</t>
         </is>
       </c>
-      <c r="B18" s="14" t="inlineStr"/>
-      <c r="C18" s="14" t="inlineStr"/>
-      <c r="D18" s="11">
-        <f> D9 − D15</f>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="8" t="n"/>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>€</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Gross Margin %</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="n"/>
+      <c r="C19" s="11" t="n"/>
+      <c r="D19" s="8">
+        <f>D18 / D9</f>
         <v/>
       </c>
-      <c r="E18" s="15" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Gross Margin %</t>
-        </is>
-      </c>
-      <c r="B19" s="14" t="inlineStr"/>
-      <c r="C19" s="14" t="inlineStr"/>
-      <c r="D19" s="11">
-        <f> D18 / D9</f>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="8" customHeight="1" s="19"/>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.  FIXED &amp; OPERATING COSTS</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="n"/>
+      <c r="C21" s="16" t="n"/>
+      <c r="D21" s="16" t="n"/>
+      <c r="E21" s="17" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Salaries (2 founders + 1 junior)</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>per month × 12</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>9200</v>
+      </c>
+      <c r="D22" s="8" t="n"/>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>€</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Studio rent (co-working space)</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>per month × 12</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="n">
+        <v>800</v>
+      </c>
+      <c r="D23" s="8" t="n"/>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>€</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Equipment depreciation (annual)</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>per month × 12</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D24" s="8" t="n"/>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>€</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Insurance &amp; admin</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>per month × 12</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>250</v>
+      </c>
+      <c r="D25" s="8" t="n"/>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>€</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    TOTAL FIXED COSTS</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="n"/>
+      <c r="C26" s="11" t="n"/>
+      <c r="D26" s="8">
+        <f>SUM(D22:D25)</f>
         <v/>
       </c>
-      <c r="E19" s="15" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="8" customHeight="1"/>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  4.  FIXED &amp; OPERATING COSTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Salaries (2 founders + 1 junior)</t>
-        </is>
-      </c>
-      <c r="B22" s="16" t="inlineStr">
-        <is>
-          <t>per month × 12</t>
-        </is>
-      </c>
-      <c r="C22" s="10" t="n">
-        <v>9200</v>
-      </c>
-      <c r="D22" s="11">
-        <f> C × 12</f>
-        <v/>
-      </c>
-      <c r="E22" s="12" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Studio rent (co-working space)</t>
-        </is>
-      </c>
-      <c r="B23" s="16" t="inlineStr">
-        <is>
-          <t>per month × 12</t>
-        </is>
-      </c>
-      <c r="C23" s="10" t="n">
-        <v>800</v>
-      </c>
-      <c r="D23" s="11">
-        <f> C × 12</f>
-        <v/>
-      </c>
-      <c r="E23" s="12" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Equipment depreciation (annual)</t>
-        </is>
-      </c>
-      <c r="B24" s="16" t="inlineStr">
-        <is>
-          <t>per month × 12</t>
-        </is>
-      </c>
-      <c r="C24" s="10" t="n">
-        <v>1200</v>
-      </c>
-      <c r="D24" s="11">
-        <f> C × 12</f>
-        <v/>
-      </c>
-      <c r="E24" s="12" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Insurance &amp; admin</t>
-        </is>
-      </c>
-      <c r="B25" s="16" t="inlineStr">
-        <is>
-          <t>per month × 12</t>
-        </is>
-      </c>
-      <c r="C25" s="10" t="n">
-        <v>250</v>
-      </c>
-      <c r="D25" s="11">
-        <f> C × 12</f>
-        <v/>
-      </c>
-      <c r="E25" s="12" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    TOTAL FIXED COSTS</t>
-        </is>
-      </c>
-      <c r="B26" s="14" t="inlineStr"/>
-      <c r="C26" s="14" t="inlineStr"/>
-      <c r="D26" s="11">
-        <f> SUM(D22:D25)</f>
-        <v/>
-      </c>
-      <c r="E26" s="15" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="8" customHeight="1"/>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>€</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="8" customHeight="1" s="19"/>
     <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+      <c r="A28" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  5.  OPERATING PROFIT (EBIT)</t>
         </is>
       </c>
+      <c r="B28" s="16" t="n"/>
+      <c r="C28" s="16" t="n"/>
+      <c r="D28" s="16" t="n"/>
+      <c r="E28" s="17" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="inlineStr">
+      <c r="A29" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">    Operating Profit (EBIT)</t>
         </is>
       </c>
-      <c r="B29" s="14" t="inlineStr"/>
-      <c r="C29" s="14" t="inlineStr"/>
-      <c r="D29" s="11">
-        <f> D18 − D26</f>
-        <v/>
-      </c>
-      <c r="E29" s="15" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="8" customHeight="1"/>
+      <c r="B29" s="11" t="n"/>
+      <c r="C29" s="11" t="n"/>
+      <c r="D29" s="8" t="n"/>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>€</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="8" customHeight="1" s="19"/>
     <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+      <c r="A31" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  6.  BREAK-EVEN ANALYSIS</t>
         </is>
       </c>
+      <c r="B31" s="16" t="n"/>
+      <c r="C31" s="16" t="n"/>
+      <c r="D31" s="16" t="n"/>
+      <c r="E31" s="17" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="9" t="inlineStr">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">    Break-Even Units / Subscribers</t>
         </is>
       </c>
-      <c r="B32" s="16" t="inlineStr">
+      <c r="B32" s="13" t="inlineStr">
         <is>
           <t>Fixed Costs ÷ (Price − Var. Cost/unit)</t>
         </is>
       </c>
-      <c r="C32" s="14" t="inlineStr"/>
-      <c r="D32" s="11">
-        <f> Fixed ÷ (Price − Var.Cost)</f>
-        <v/>
-      </c>
-      <c r="E32" s="12" t="inlineStr">
+      <c r="C32" s="11" t="n"/>
+      <c r="D32" s="8" t="n"/>
+      <c r="E32" s="9" t="inlineStr">
         <is>
           <t>units</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="8" customHeight="1"/>
+    <row r="33" ht="8" customHeight="1" s="19"/>
     <row r="34">
-      <c r="A34" s="7" t="inlineStr">
+      <c r="A34" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">  📌 Company context: Aura Motion is a creative services agency — COGS are mainly freelancer costs and per-project assets. Retainer clients provide predictable monthly revenue.</t>
         </is>

</xml_diff>